<commit_message>
0.4b - Corpus: pérdidas, JPEG y GIF, inmovilizado y documentos grandes
Claude-Session: https://claude.ai/code/session_014nGJQXvTkbMhTYikVkHfor
</commit_message>
<xml_diff>
--- a/tests/ficheros/calc/formulas.xlsx
+++ b/tests/ficheros/calc/formulas.xlsx
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B16" s="4" t="n">
         <f aca="true">NOW()</f>
-        <v>46320.092829782</v>
+        <v>46320.0959064359</v>
       </c>
     </row>
   </sheetData>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="B9" s="0" t="n">
         <f aca="true">RAND()</f>
-        <v>0.535200671806533</v>
+        <v>0.799331247850831</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
0.5 - tools/volcar_lo.py: volcado de referencia del corpus por UNO; corpus en en-US
Claude-Session: https://claude.ai/code/session_014nGJQXvTkbMhTYikVkHfor
</commit_message>
<xml_diff>
--- a/tests/ficheros/calc/formulas.xlsx
+++ b/tests/ficheros/calc/formulas.xlsx
@@ -206,9 +206,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="&quot;VERDADERO&quot;;&quot;VERDADERO&quot;;&quot;FALSO&quot;"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yy\ hh:mm"/>
+    <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yy\ hh:mm\ AM/PM"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -609,7 +609,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -750,7 +750,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -900,7 +900,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B19" s="0" t="str">
         <f aca="false">TEXT(1234.5,"#,##0.00")</f>
-        <v>1.234,50</v>
+        <v>1,234.50</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1077,7 +1077,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -1212,13 +1212,13 @@
       </c>
       <c r="B16" s="4" t="n">
         <f aca="true">NOW()</f>
-        <v>46320.0959064359</v>
+        <v>46320.0988555863</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -1341,7 +1341,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -1464,7 +1464,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="B9" s="0" t="n">
         <f aca="true">RAND()</f>
-        <v>0.799331247850831</v>
+        <v>0.874154076953715</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10599,7 +10599,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>

</xml_diff>